<commit_message>
auto: snapshot 2026-07-25 05:30:39
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -463,11 +463,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-25 13:00:12</t>
+          <t>Timestamp: 2026-07-25 13:30:38</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>720</v>
       </c>
     </row>
     <row r="3">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>14213</v>
+        <v>14333</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>18229</v>
+        <v>18349</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>17344</v>
+        <v>17584</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>9506</v>
+        <v>9626</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>8695</v>
+        <v>8815</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:30:22
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -1352,11 +1352,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:00:09</t>
+          <t>Timestamp: 2026-07-26 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>33995</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="3">
@@ -1773,11 +1773,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>19202</v>
+        <v>19442</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+4869</t>
+          <t>+5109</t>
         </is>
       </c>
     </row>
@@ -1788,11 +1788,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>23365</v>
+        <v>23725</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+5016</t>
+          <t>+5376</t>
         </is>
       </c>
     </row>
@@ -1833,11 +1833,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>22877</v>
+        <v>23237</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+5293</t>
+          <t>+5653</t>
         </is>
       </c>
     </row>
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>15003</v>
+        <v>15243</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+5377</t>
+          <t>+5617</t>
         </is>
       </c>
     </row>
@@ -2148,11 +2148,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>11095</v>
+        <v>11178</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2280</t>
+          <t>+2363</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:44:29
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -1352,11 +1352,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:30:21</t>
+          <t>Timestamp: 2026-07-26 13:44:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1283</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="3">
@@ -1773,11 +1773,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>19442</v>
+        <v>19562</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+5109</t>
+          <t>+5229</t>
         </is>
       </c>
     </row>
@@ -2148,11 +2148,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>11178</v>
+        <v>11603</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2363</t>
+          <t>+2788</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:06:08
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -2241,11 +2241,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-27 13:00:10</t>
+          <t>Timestamp: 2026-07-27 13:06:07</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>31943</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:28:31
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3130,11 +3130,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:00:09</t>
+          <t>Timestamp: 2026-07-28 13:28:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>24578</v>
+        <v>24634</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1008</t>
+          <t>+1064</t>
         </is>
       </c>
     </row>
@@ -3566,11 +3566,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>35318</v>
+        <v>35402</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+4161</t>
+          <t>+4245</t>
         </is>
       </c>
     </row>
@@ -3866,11 +3866,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>30856</v>
+        <v>30940</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3805</t>
+          <t>+3889</t>
         </is>
       </c>
     </row>
@@ -3956,11 +3956,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>3333</v>
+        <v>3417</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3313</t>
+          <t>+3397</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:30:20
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3130,11 +3130,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:28:30</t>
+          <t>Timestamp: 2026-07-28 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>308</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>24634</v>
+        <v>24662</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1064</t>
+          <t>+1092</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:58:50
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3130,11 +3130,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:30:20</t>
+          <t>Timestamp: 2026-07-28 13:58:49</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>336</v>
+        <v>756</v>
       </c>
     </row>
     <row r="3">
@@ -3566,11 +3566,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>35402</v>
+        <v>35486</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+4245</t>
+          <t>+4329</t>
         </is>
       </c>
     </row>
@@ -3611,11 +3611,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>29733</v>
+        <v>29901</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1512</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -3866,11 +3866,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>30940</v>
+        <v>31024</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3889</t>
+          <t>+3973</t>
         </is>
       </c>
     </row>
@@ -3956,11 +3956,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>3417</v>
+        <v>3501</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3397</t>
+          <t>+3481</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:27:23
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4019,11 +4019,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:00:09</t>
+          <t>Timestamp: 2026-07-29 13:27:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3">
@@ -4305,11 +4305,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>8848</v>
+        <v>8968</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+1224</t>
+          <t>+1344</t>
         </is>
       </c>
     </row>
@@ -4500,11 +4500,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>32643</v>
+        <v>32763</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2742</t>
+          <t>+2862</t>
         </is>
       </c>
     </row>
@@ -4755,11 +4755,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>34490</v>
+        <v>34550</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3466</t>
+          <t>+3526</t>
         </is>
       </c>
     </row>
@@ -4845,11 +4845,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>6671</v>
+        <v>6851</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3170</t>
+          <t>+3350</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:57:35
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4019,11 +4019,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:30:20</t>
+          <t>Timestamp: 2026-07-29 13:57:34</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>480</v>
+        <v>600</v>
       </c>
     </row>
     <row r="3">
@@ -4755,11 +4755,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>34550</v>
+        <v>34610</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3526</t>
+          <t>+3586</t>
         </is>
       </c>
     </row>
@@ -4845,11 +4845,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>6851</v>
+        <v>6911</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3350</t>
+          <t>+3410</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:00:09
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4875,4 +4876,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-30 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>16876</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>152</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5379</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>10390</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1422</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6368</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4749</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>29078</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>41486</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2595</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>35343</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2580</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3366</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2040</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21027</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>37370</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2760</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>15217</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>9110</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2199</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:00:05
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -13,6 +13,7 @@
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5764,4 +5765,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-31 13:00:04</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>10532</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5670</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+291</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11660</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1270</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6668</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>30908</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1830</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>44294</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2748</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>37122</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1779</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3366</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21037</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>40070</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2640</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>15733</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+516</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>11669</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2499</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1262</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+311</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:30:16
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -5797,11 +5797,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-31 13:00:04</t>
+          <t>Timestamp: 2026-07-31 13:30:15</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10532</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3">
@@ -6218,11 +6218,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>30908</v>
+        <v>30968</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1830</t>
+          <t>+1890</t>
         </is>
       </c>
     </row>
@@ -6233,11 +6233,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>44294</v>
+        <v>44354</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+2748</t>
+          <t>+2808</t>
         </is>
       </c>
     </row>
@@ -6278,11 +6278,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>37122</v>
+        <v>37182</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1779</t>
+          <t>+1839</t>
         </is>
       </c>
     </row>
@@ -6533,11 +6533,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>40070</v>
+        <v>40130</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2640</t>
+          <t>+2700</t>
         </is>
       </c>
     </row>
@@ -6623,11 +6623,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>11669</v>
+        <v>11729</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+2499</t>
+          <t>+2559</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:00:10
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6653,4 +6654,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-01 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12526</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5970</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6968</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45854</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39162</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21799</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+762</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>41993</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+1863</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>16784</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1051</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+1890</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1262</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:00:09
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7542,4 +7543,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-02 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>17860</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>282</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+120</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6570</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1793</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1793</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>7568</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45874</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>1376</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1376</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>3584</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+2039</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>23163</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1364</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>45602</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3609</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>21303</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+4119</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:30:22
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -7575,11 +7575,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-02 13:00:09</t>
+          <t>Timestamp: 2026-08-02 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>17860</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3">
@@ -8311,11 +8311,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>45602</v>
+        <v>45722</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3609</t>
+          <t>+3729</t>
         </is>
       </c>
     </row>
@@ -8371,11 +8371,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>21303</v>
+        <v>21427</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+4119</t>
+          <t>+4243</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -16,6 +16,7 @@
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1329,6 +1330,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-03 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22641</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>582</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>7290</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>5399</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3606</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>8168</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>46714</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>4123</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+2747</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7304</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+3720</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24344</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>50729</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+5007</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>25103</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3676</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:30:23
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -1360,11 +1360,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:00:10</t>
+          <t>Timestamp: 2026-08-03 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>22641</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>5399</v>
+        <v>5459</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3606</t>
+          <t>+3666</t>
         </is>
       </c>
     </row>
@@ -1886,11 +1886,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>7304</v>
+        <v>7364</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+3720</t>
+          <t>+3780</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:30:24
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -2249,11 +2249,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:00:09</t>
+          <t>Timestamp: 2026-08-04 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10516</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -2985,11 +2985,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>53004</v>
+        <v>53064</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2335</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:30:21
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3138,11 +3138,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-05 13:00:10</t>
+          <t>Timestamp: 2026-08-05 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>11472</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3">
@@ -3874,11 +3874,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>55884</v>
+        <v>55944</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2820</t>
+          <t>+2880</t>
         </is>
       </c>
     </row>
@@ -3964,11 +3964,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>14819</v>
+        <v>15079</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1460</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:00:09
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -19,6 +19,7 @@
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3996,6 +3997,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-06 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>17096</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1452</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>9068</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>47746</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+672</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1737</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>16851</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+1608</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24354</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>59004</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3060</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>32444</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2976</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>18091</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3012</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:18:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4027,11 +4027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:00:09</t>
+          <t>Timestamp: 2026-08-06 13:18:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>17096</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3">
@@ -4703,11 +4703,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>16851</v>
+        <v>16911</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1608</t>
+          <t>+1668</t>
         </is>
       </c>
     </row>
@@ -4763,11 +4763,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>59004</v>
+        <v>59054</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3060</t>
+          <t>+3110</t>
         </is>
       </c>
     </row>
@@ -4823,11 +4823,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>32444</v>
+        <v>32504</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2976</t>
+          <t>+3036</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:30:24
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4027,11 +4027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:18:26</t>
+          <t>Timestamp: 2026-08-06 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>170</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3">
@@ -4463,11 +4463,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>47746</v>
+        <v>47806</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+672</t>
+          <t>+732</t>
         </is>
       </c>
     </row>
@@ -4853,11 +4853,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>18091</v>
+        <v>18151</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3012</t>
+          <t>+3072</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:48:43
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4027,11 +4027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:30:23</t>
+          <t>Timestamp: 2026-08-06 13:48:42</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>290</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -4703,11 +4703,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>16911</v>
+        <v>16971</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1668</t>
+          <t>+1728</t>
         </is>
       </c>
     </row>
@@ -4763,11 +4763,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>59054</v>
+        <v>59124</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3110</t>
+          <t>+3180</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20,6 +20,7 @@
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4885,6 +4886,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-07 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>15147</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>9908</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>48366</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>20222</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3251</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24354</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>62816</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3692</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>35201</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2697</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>21836</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3685</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:29:39
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4916,11 +4916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:00:12</t>
+          <t>Timestamp: 2026-08-07 13:29:39</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>15147</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
@@ -5592,11 +5592,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>20222</v>
+        <v>20282</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3251</t>
+          <t>+3311</t>
         </is>
       </c>
     </row>
@@ -5652,11 +5652,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>62816</v>
+        <v>62876</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3692</t>
+          <t>+3752</t>
         </is>
       </c>
     </row>
@@ -5682,11 +5682,11 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>2060</v>
+        <v>2070</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+10</t>
         </is>
       </c>
     </row>
@@ -5712,11 +5712,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>35201</v>
+        <v>35261</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2697</t>
+          <t>+2757</t>
         </is>
       </c>
     </row>
@@ -5742,11 +5742,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>21836</v>
+        <v>21896</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3685</t>
+          <t>+3745</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:59:56
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4916,11 +4916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:30:29</t>
+          <t>Timestamp: 2026-08-07 13:59:55</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>250</v>
+        <v>730</v>
       </c>
     </row>
     <row r="3">
@@ -5052,11 +5052,11 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>8310</v>
+        <v>8610</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -5592,11 +5592,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>20282</v>
+        <v>20342</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3311</t>
+          <t>+3371</t>
         </is>
       </c>
     </row>
@@ -5652,11 +5652,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>62876</v>
+        <v>62936</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3752</t>
+          <t>+3812</t>
         </is>
       </c>
     </row>
@@ -5742,11 +5742,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>21896</v>
+        <v>21956</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3745</t>
+          <t>+3805</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:30:29
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -5805,11 +5805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:00:11</t>
+          <t>Timestamp: 2026-08-08 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>18324</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3">
@@ -6481,11 +6481,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>23025</v>
+        <v>23145</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2683</t>
+          <t>+2803</t>
         </is>
       </c>
     </row>
@@ -6541,11 +6541,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>65906</v>
+        <v>66026</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2970</t>
+          <t>+3090</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:37:22
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -5805,11 +5805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:30:28</t>
+          <t>Timestamp: 2026-08-08 13:37:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>240</v>
+        <v>461</v>
       </c>
     </row>
     <row r="3">
@@ -6601,11 +6601,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>37509</v>
+        <v>37730</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2248</t>
+          <t>+2469</t>
         </is>
       </c>
     </row>

</xml_diff>